<commit_message>
mise a jour xls avec photo pepe
</commit_message>
<xml_diff>
--- a/data/Genealogie_MEME.xlsx
+++ b/data/Genealogie_MEME.xlsx
@@ -847,6 +847,15 @@
   </si>
   <si>
     <t>https://i.postimg.cc/gkvkD0fy/Photo-MEME.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/KjSVSDs0/homme-inconnu.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/MH242mr3/femme-inconnue.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/TPQYPpXc/Photo-PEPE.png</t>
   </si>
 </sst>
 </file>
@@ -7458,6 +7467,9 @@
       <c r="T3" s="17"/>
       <c r="U3" s="17"/>
       <c r="V3" s="17"/>
+      <c r="W3" s="16" t="s">
+        <v>279</v>
+      </c>
     </row>
     <row r="4" customFormat="1" s="16">
       <c r="A4" s="17" t="s">
@@ -7509,6 +7521,9 @@
       <c r="U4" s="17"/>
       <c r="V4" s="17" t="s">
         <v>264</v>
+      </c>
+      <c r="W4" s="16" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="5" customFormat="1" s="16">
@@ -7550,7 +7565,9 @@
       <c r="T5" s="17"/>
       <c r="U5" s="17"/>
       <c r="V5" s="17"/>
-      <c r="W5" s="17"/>
+      <c r="W5" s="17" t="s">
+        <v>277</v>
+      </c>
     </row>
     <row r="6" customFormat="1" s="16">
       <c r="A6" s="17" t="s">
@@ -7593,7 +7610,9 @@
       <c r="T6" s="17"/>
       <c r="U6" s="17"/>
       <c r="V6" s="17"/>
-      <c r="W6" s="17"/>
+      <c r="W6" s="17" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="7" customFormat="1" s="16">
       <c r="A7" s="17" t="s">
@@ -7640,7 +7659,9 @@
       <c r="T7" s="17"/>
       <c r="U7" s="17"/>
       <c r="V7" s="17"/>
-      <c r="W7" s="17"/>
+      <c r="W7" s="17" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="8" customFormat="1" s="16">
       <c r="A8" s="17" t="s">
@@ -7685,7 +7706,9 @@
       <c r="T8" s="17"/>
       <c r="U8" s="17"/>
       <c r="V8" s="17"/>
-      <c r="W8" s="17"/>
+      <c r="W8" s="17" t="s">
+        <v>277</v>
+      </c>
     </row>
     <row r="9" customFormat="1" s="16">
       <c r="A9" s="17" t="s">
@@ -7737,7 +7760,7 @@
         <v>224</v>
       </c>
       <c r="W9" s="24" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10" customFormat="1" s="16">
@@ -7790,7 +7813,7 @@
         <v>231</v>
       </c>
       <c r="W10" s="24" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" customFormat="1" s="16">
@@ -7841,7 +7864,7 @@
         <v>230</v>
       </c>
       <c r="W11" s="24" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="12" customFormat="1" s="16">
@@ -7892,7 +7915,7 @@
         <v>229</v>
       </c>
       <c r="W12" s="24" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" customFormat="1" s="16">
@@ -7945,7 +7968,7 @@
         <v>228</v>
       </c>
       <c r="W13" s="24" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14" customFormat="1" s="16">
@@ -7996,7 +8019,7 @@
         <v>232</v>
       </c>
       <c r="W14" s="24" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="15" customFormat="1" s="16">
@@ -8051,7 +8074,7 @@
         <v>252</v>
       </c>
       <c r="W15" s="24" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="16" customFormat="1" s="16">
@@ -8096,7 +8119,7 @@
       <c r="U16" s="17"/>
       <c r="V16" s="17"/>
       <c r="W16" s="24" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="17" customFormat="1" s="16">
@@ -8141,7 +8164,7 @@
       <c r="U17" s="17"/>
       <c r="V17" s="17"/>
       <c r="W17" s="24" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="18" customFormat="1" s="16">

</xml_diff>

<commit_message>
lien elise piste recherche
</commit_message>
<xml_diff>
--- a/data/Genealogie_MEME.xlsx
+++ b/data/Genealogie_MEME.xlsx
@@ -774,6 +774,15 @@
   </si>
   <si>
     <t>époux d'une tatan du PEPE</t>
+  </si>
+  <si>
+    <t>Simone Cyprienne Victoria</t>
+  </si>
+  <si>
+    <t>Quelle liens avec les autres LAULAGNIER?</t>
+  </si>
+  <si>
+    <t>Quelle liens avec les autres LAULAGNIER? (n'apparait pas dans l'acte notarié donc peu probable fratrie, reste soeur de Francois?</t>
   </si>
 </sst>
 </file>
@@ -1353,7 +1362,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20.08984375" customWidth="1" min="2" max="2" bestFit="1"/>
+    <col width="22.6328125" customWidth="1" min="2" max="2" bestFit="1"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4" bestFit="1"/>
     <col width="8" customWidth="1" min="5" max="5"/>
@@ -1693,7 +1702,7 @@
         <v>157</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>172</v>
+        <v>253</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>30</v>
@@ -2082,7 +2091,9 @@
       <c r="O16" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="P16" s="4"/>
+      <c r="P16" s="4" t="s">
+        <v>255</v>
+      </c>
       <c r="Q16" s="4" t="s">
         <v>63</v>
       </c>

</xml_diff>